<commit_message>
CRUD-MONEDA - BIOMETRICO Y REGLAS FALTA MEJORAR Y RETOCAR
</commit_message>
<xml_diff>
--- a/marcajes.xlsx
+++ b/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="74">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -224,6 +224,15 @@
   </si>
   <si>
     <t>26/08/2026, 01:56:21 p. m.</t>
+  </si>
+  <si>
+    <t>24765865</t>
+  </si>
+  <si>
+    <t>LUIS ROJAS</t>
+  </si>
+  <si>
+    <t>29/08/2026, 02:06:46 p. m.</t>
   </si>
 </sst>
 </file>
@@ -612,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1557,6 +1566,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" t="s">
+        <v>73</v>
+      </c>
+      <c r="D56" t="s">
+        <v>8</v>
+      </c>
+      <c r="E56" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
CRUD DE TASAS Y MONEDAS LISTAS MEJORAS EN EL BIOMETRICO YA SACA TODAS LAS PERSONAS DEL BIOMETRICO Y NO POR PAGINACION FALTA AJUSTAR LO DE LOS DIAS LIBRES Y PERMISOS
</commit_message>
<xml_diff>
--- a/marcajes.xlsx
+++ b/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="81">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -233,6 +233,27 @@
   </si>
   <si>
     <t>29/08/2026, 02:06:46 p. m.</t>
+  </si>
+  <si>
+    <t>29/08/2026, 03:00:06 p. m.</t>
+  </si>
+  <si>
+    <t>29/08/2026, 03:59:44 p. m.</t>
+  </si>
+  <si>
+    <t>29/08/2026, 03:59:53 p. m.</t>
+  </si>
+  <si>
+    <t>30/08/2026, 08:28:33 a. m.</t>
+  </si>
+  <si>
+    <t>31/08/2026, 09:52:04 a. m.</t>
+  </si>
+  <si>
+    <t>31/08/2026, 11:58:58 a. m.</t>
+  </si>
+  <si>
+    <t>31/08/2026, 05:33:41 p. m.</t>
   </si>
 </sst>
 </file>
@@ -621,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1583,6 +1604,125 @@
         <v>9</v>
       </c>
     </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>71</v>
+      </c>
+      <c r="B57" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" t="s">
+        <v>74</v>
+      </c>
+      <c r="D57" t="s">
+        <v>8</v>
+      </c>
+      <c r="E57" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>11</v>
+      </c>
+      <c r="B58" t="s">
+        <v>12</v>
+      </c>
+      <c r="C58" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>17</v>
+      </c>
+      <c r="B59" t="s">
+        <v>18</v>
+      </c>
+      <c r="C59" t="s">
+        <v>76</v>
+      </c>
+      <c r="D59" t="s">
+        <v>8</v>
+      </c>
+      <c r="E59" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60" t="s">
+        <v>12</v>
+      </c>
+      <c r="C60" t="s">
+        <v>77</v>
+      </c>
+      <c r="D60" t="s">
+        <v>8</v>
+      </c>
+      <c r="E60" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>17</v>
+      </c>
+      <c r="B61" t="s">
+        <v>18</v>
+      </c>
+      <c r="C61" t="s">
+        <v>78</v>
+      </c>
+      <c r="D61" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>11</v>
+      </c>
+      <c r="B62" t="s">
+        <v>12</v>
+      </c>
+      <c r="C62" t="s">
+        <v>79</v>
+      </c>
+      <c r="D62" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>11</v>
+      </c>
+      <c r="B63" t="s">
+        <v>12</v>
+      </c>
+      <c r="C63" t="s">
+        <v>80</v>
+      </c>
+      <c r="D63" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
correcciones en horarios- dias libres voy agregar una nueva regla para validar horas diurnas y nocturnas
</commit_message>
<xml_diff>
--- a/marcajes.xlsx
+++ b/marcajes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="85">
   <si>
     <t>ID / Cédula</t>
   </si>
@@ -254,6 +254,18 @@
   </si>
   <si>
     <t>31/08/2026, 05:33:41 p. m.</t>
+  </si>
+  <si>
+    <t>01/09/2026, 10:54:51 a. m.</t>
+  </si>
+  <si>
+    <t>22652518</t>
+  </si>
+  <si>
+    <t>JORWINS MARCANO</t>
+  </si>
+  <si>
+    <t>01/09/2026, 10:55:51 a. m.</t>
   </si>
 </sst>
 </file>
@@ -642,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1723,6 +1735,40 @@
         <v>9</v>
       </c>
     </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>17</v>
+      </c>
+      <c r="B64" t="s">
+        <v>18</v>
+      </c>
+      <c r="C64" t="s">
+        <v>81</v>
+      </c>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>82</v>
+      </c>
+      <c r="B65" t="s">
+        <v>83</v>
+      </c>
+      <c r="C65" t="s">
+        <v>84</v>
+      </c>
+      <c r="D65" t="s">
+        <v>8</v>
+      </c>
+      <c r="E65" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>